<commit_message>
fix(business-plans-en-2): Restaurant y Bakery regenerados con la ronda de arreglos — gates G1-G9 en verde, cifras del caso intactas
astro-site/public/dl/restaurant-business-plan/{restaurant-business-plan.docx,restaurant-financial-projections.xlsx,restaurant-opening-checklist.xlsx}
y astro-site/public/dl/bakery-business-plan/{bakery-business-plan.docx,bakery-financial-projections.xlsx,bakery-opening-checklist.xlsx}
(VPS, sha256 iguales); scripts/productos-digitales/business-plans-en-2/textos_es.json y censo_es.json re-extraídos por
las 5 celdas nuevas de POR_CELDA; textos_en/GREST.json (notas F17/F60 acortadas). Caché numérica y cifras_caso.json
sin cambios; regresión FT/CAF 6/6 idéntica en canónico. §8 en scripts/productos-digitales/business-plans-en-2/F2-NOTAS.md.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hr4gADNsFqH4pKHsfukJDM
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
+++ b/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cost of coffee and beverages against their own sales: inside the 25-30% that the industry benchmarks table on the "Instructions" tab gives for coffee (kit estimate)</t>
+          <t>Cost of coffee and beverages against their own sales: inside the 20-30% that the industry benchmarks table on the "Instructions" tab gives for coffee (kit estimate)</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
-          <t>Artisan bread and pastries from the shop, plus the wholesale channel to cafés and restaurants (the bread you sell to another business is the same product line as the bread you sell at the counter; only the channel changes). NOTE: the model projects sales with ONE engine — transactions × average check × days — so a delivery to another business enters here as one more transaction, not as a big order. What the workbook does capture is its effect on cash, through the average collection days on "0. Assumptions". If wholesale weighs heavily in your project, model it separately · The percentage on the right ("Tax-exempt share of the line (%)") is the part of this line that carries no sales tax: bakery goods to go, plus wholesale sales to a café that resells them (with a resale certificate on file). The example is 0.80. Many states exempt bakery goods sold to go and tax what is eaten in the shop (California, for instance, does so with its 80/80 rule): check your state. At 0 the workbook taxes the whole line. In the UK, cold bakery goods to go are zero-rated and on-site consumption carries 20% VAT. It only affects cash flow: the P&amp;L is excl. sales tax</t>
+          <t>Artisan bread and pastries from the shop, plus the wholesale channel to cafés and restaurants (the bread you sell to another business is the same product line as the bread you sell at the counter; only the channel changes). NOTE: the model projects sales with ONE engine — transactions × average check × days — so a delivery to another business enters here as one more transaction, not as a big order. What the workbook does capture is its effect on cash, through the average collection days on "0. Assumptions". If wholesale weighs heavily in your project, model it separately · The percentage on the right ("Tax-exempt share of the line (%)") is the part of this line that carries no sales tax: bakery goods to go, plus wholesale sales to a café that resells them (with a resale certificate on file). The example is 0.80. Many states exempt bakery goods sold to go and tax what is eaten in the shop, but the rules vary by state: check yours. At 0 the workbook taxes the whole line. In the UK, cold bakery goods to go are zero-rated and on-site consumption carries 20% VAT. It only affects cash flow: the P&amp;L is excl. sales tax</t>
         </is>
       </c>
       <c r="G10" s="67">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="J21" s="33" t="inlineStr">
         <is>
-          <t>Average number of people at the counter at the same time through the day: one fixed person plus reinforcement for the morning and afternoon peaks</t>
+          <t>Average number of people at the counter at the same time through the day: two in this example, which covers the morning and afternoon peaks and the coffee corner</t>
         </is>
       </c>
     </row>
@@ -5787,7 +5787,7 @@
       </c>
       <c r="J23" s="33" t="inlineStr">
         <is>
-          <t>The head baker alone. If your bakery starts with two people, raise it here</t>
+          <t>The head baker and the baker. Change it if your production shift has a different number of people</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6559,7 @@
       </c>
       <c r="D46" s="17" t="inlineStr">
         <is>
-          <t>Year 2 is kept moderate, which is the prudent choice, but not lower: it is the year when loan repayment weighs the most, and with less growth the cushion over the cash break-even would fall below the 15% this workbook asks for.</t>
+          <t>Year 2 is kept moderate, which is the prudent choice, but not lower: with less growth the cushion over the cash break-even would fall below the 15% this workbook asks for.</t>
         </is>
       </c>
     </row>
@@ -6581,7 +6581,7 @@
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>The counter is paid at the time of sale, but a café or restaurant that buys from you usually pays on terms, often 30 days. With the weight this business gives to wholesale, the weighted average is a few days, and the "12-Month Cash Flow" tab already takes it into account.</t>
+          <t>The counter is paid at the time of sale, but a café or restaurant that buys from you usually pays on terms, often 30 days. With the weight this business gives to wholesale, the weighted average is about a day, and the "12-Month Cash Flow" tab already takes it into account.</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6962,7 @@
       </c>
       <c r="D66" s="17" t="inlineStr">
         <is>
-          <t>This workbook does not copy a payback from anyone: it calculates it with ITS investment and ITS cash flows before debt, and publishes it in the figures block, in the "Project payback (years), before debt" row. A bakery takes longer to pay back its investment than a coffee shop, because the oven, the mixer and the coolers are paid for on day one</t>
+          <t>This workbook does not copy a payback from anyone: it calculates it with ITS investment and ITS cash flows before debt, and publishes it in the figures block, in the "Project payback (years), before debt" row.</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>SBA Microloans go up to $50,000 through nonprofit intermediaries. Like row 8, a source of funds only: not in the schedule or the DSCR. If it is your only loan, enter it in row 7 instead</t>
+          <t>SBA Microloans go up to 50,000 through nonprofit intermediaries. Like row 8, a source of funds only: not in the schedule or the DSCR. If it is your only loan, enter it in row 7 instead</t>
         </is>
       </c>
       <c r="D9" s="28" t="n"/>

</xml_diff>

<commit_message>
Arreglos sin correo en 39 xlsx LIVE: literales > 255 (Excel reparaba el libro), desplegable ✓/☐/N/A, nota de la holgura, ITC del gas (Taquería), nota trimestral EN
Parche XML con scripts/productos-digitales/parche_xml_xlsx.py --apply (solo el contenido de las celdas que cambian;
cachés intactas). Verificación celda a celda contra el respaldo: 76 celdas troceadas, 42 con texto nuevo, 0 cambios
fuera de regla; gate LIT255 verde en los 753 xlsx de dl/. Prueba A/B en Excel: el original perdía la fórmula de
Inversión Inicial!D27 al repararse; el parcheado abre sin reparar y con la fórmula viva.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
+++ b/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
@@ -2230,7 +2230,7 @@
         <v>0.023996190604741497</v>
       </c>
       <c r="D28" t="str">
-        <f>IFERROR("At "&amp;TEXT('0. Assumptions'!$B$55,"0%")&amp;" of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a build-out without a cushion: the percentage is in ""0. Assumptions""","")</f>
+        <f>IFERROR("At "&amp;TEXT('0. Assumptions'!$B$55,"0%")&amp;" of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a "&amp;"build-out without a cushion: the percentage is in ""0. Assumptions""","")</f>
         <v>At 10% of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a build-out without a cushion: the percentage is in "0. Assumptions"</v>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="O20" s="28" t="inlineStr">
         <is>
-          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly (April, July, October, January): if your state requires monthly filing, expect smaller payments every month instead</t>
+          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly, in the month after each plan quarter (Months 4, 7 and 10, and the fourth quarter in Month 13: April, July, October and January when Month 1 is January): if your state requires monthly filing, expect smaller payments every month instead</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ronda 2 en los xlsx LIVE: holgura y 4.º trimestre EN (10+10+11), B67 contra la holgura de caja (16)
parche_xml_xlsx.py --apply sobre dl/: 30 ficheros; verificación acumulada contra el respaldo VERDE (41 ficheros, 76 celdas
troceadas, 73 con texto nuevo); gate LIT255 VERDE; gates_en.py --solo G1 (business-plans-en) VERDE con los ES troceados.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
+++ b/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>How far you can fall below plan before you start losing money</t>
+          <t>How far planned sales must sit above cash break-even (fixed costs and the loan payment). The drop you can absorb is somewhat smaller: with a 15% cushion, about 13% of plan</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="E24" s="28" t="inlineStr">
         <is>
-          <t>How far you can fall before you cannot pay the fixed costs and the loan payment. The required minimum is set in the "0. Assumptions" tab</t>
+          <t>How far planned sales sit above cash break-even. The drop you can absorb before you cannot pay the fixed costs and the loan payment is somewhat smaller: with a 25% cushion, 20%. The required minimum is set in the "0. Assumptions" tab</t>
         </is>
       </c>
       <c r="F24" s="28" t="n"/>
@@ -8441,7 +8441,7 @@
     <row r="34" ht="134.75" customHeight="1">
       <c r="A34" s="46" t="inlineStr">
         <is>
-          <t>Fourth-quarter sales tax is settled in January of the following year, so it does not appear in this table. The model pays year-1 income tax in July of year 2 (a simplification: estimated tax payments are usually quarterly). The loan payment is spread in twelve equal parts following the ANNUAL schedule in the Financing tab, and payroll in twelve monthly installments (plus extra pay periods in their month, only if pay periods &gt; 12).</t>
+          <t>Fourth-quarter sales tax is settled in Month 13 (January of the following year when Month 1 is January), so it does not appear in this table. The model pays year-1 income tax in July of year 2 (a simplification: estimated tax payments are usually quarterly). The loan payment is spread in twelve equal parts following the ANNUAL schedule in the Financing tab, and payroll in twelve monthly installments (plus extra pay periods in their month, only if pay periods &gt; 12).</t>
         </is>
       </c>
       <c r="B34" s="28" t="n"/>

</xml_diff>

<commit_message>
Tanda de arreglos sin correo (30-oct): literales > 255 que Excel reparaba, desplegable ✓/☐/N/A, holgura, ITC del gas, notas EN (#186)
41 xlsx LIVE por parche XML + 3 documentos de guía regenerados; fuente al día (inject_cache trocea, circuito EN funde, gate parche_xml_xlsx.py --check). Detalle: SESSION_HANDOFF_2026-10-30-tanda-arreglos.md.

Via: Claude Code

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
+++ b/astro-site/public/dl/bakery-business-plan/bakery-financial-projections.xlsx
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>How far you can fall below plan before you start losing money</t>
+          <t>How far planned sales must sit above cash break-even (fixed costs and the loan payment). The drop you can absorb is somewhat smaller: with a 15% cushion, about 13% of plan</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
         <v>0.023996190604741497</v>
       </c>
       <c r="D28" t="str">
-        <f>IFERROR("At "&amp;TEXT('0. Assumptions'!$B$55,"0%")&amp;" of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a build-out without a cushion: the percentage is in ""0. Assumptions""","")</f>
+        <f>IFERROR("At "&amp;TEXT('0. Assumptions'!$B$55,"0%")&amp;" of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a "&amp;"build-out without a cushion: the percentage is in ""0. Assumptions""","")</f>
         <v>At 10% of the BUILD-OUT items of this block (architect and building permits, construction, electrical service upgrade for the ovens, oven ventilation and exhaust, signage), not of the whole block: the other items are left out. No lender funds a build-out without a cushion: the percentage is in "0. Assumptions"</v>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="E24" s="28" t="inlineStr">
         <is>
-          <t>How far you can fall before you cannot pay the fixed costs and the loan payment. The required minimum is set in the "0. Assumptions" tab</t>
+          <t>How far planned sales sit above cash break-even. The drop you can absorb before you cannot pay the fixed costs and the loan payment is somewhat smaller: with a 25% cushion, 20%. The required minimum is set in the "0. Assumptions" tab</t>
         </is>
       </c>
       <c r="F24" s="28" t="n"/>
@@ -8027,7 +8027,7 @@
       </c>
       <c r="O20" s="28" t="inlineStr">
         <is>
-          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly (April, July, October, January): if your state requires monthly filing, expect smaller payments every month instead</t>
+          <t>Cash only leaves when the quarter's result is positive. Months without a settlement are left blank, not zero. The cell turns RED when the payment takes more cash than is left that month. The model settles quarterly, in the month after each plan quarter (Months 4, 7 and 10, and the fourth quarter in Month 13: April, July, October and January when Month 1 is January): if your state requires monthly filing, expect smaller payments every month instead</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
     <row r="34" ht="134.75" customHeight="1">
       <c r="A34" s="46" t="inlineStr">
         <is>
-          <t>Fourth-quarter sales tax is settled in January of the following year, so it does not appear in this table. The model pays year-1 income tax in July of year 2 (a simplification: estimated tax payments are usually quarterly). The loan payment is spread in twelve equal parts following the ANNUAL schedule in the Financing tab, and payroll in twelve monthly installments (plus extra pay periods in their month, only if pay periods &gt; 12).</t>
+          <t>Fourth-quarter sales tax is settled in Month 13 (January of the following year when Month 1 is January), so it does not appear in this table. The model pays year-1 income tax in July of year 2 (a simplification: estimated tax payments are usually quarterly). The loan payment is spread in twelve equal parts following the ANNUAL schedule in the Financing tab, and payroll in twelve monthly installments (plus extra pay periods in their month, only if pay periods &gt; 12).</t>
         </is>
       </c>
       <c r="B34" s="28" t="n"/>

</xml_diff>